<commit_message>
feat(expenses): logically align demo excel workbook with actual spend modal 13 tasks and 6 subcategories
</commit_message>
<xml_diff>
--- a/frontend/public/sample-docs/73 Broadway - Expense Tracker.xlsx
+++ b/frontend/public/sample-docs/73 Broadway - Expense Tracker.xlsx
@@ -4,12 +4,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Total Expenses" sheetId="1" r:id="rId1"/>
-    <sheet name="Construction Exp" sheetId="2" r:id="rId2"/>
-    <sheet name="Labour Exp" sheetId="3" r:id="rId3"/>
-    <sheet name="Accounting &amp; Legal fee" sheetId="4" r:id="rId4"/>
-    <sheet name="Bank Fee" sheetId="5" r:id="rId5"/>
-    <sheet name="Municipal Exp" sheetId="6" r:id="rId6"/>
-    <sheet name="Misc Exp" sheetId="7" r:id="rId7"/>
+    <sheet name="Soft Costs" sheetId="2" r:id="rId2"/>
+    <sheet name="Municipal &amp; Permits" sheetId="3" r:id="rId3"/>
+    <sheet name="Sitework &amp; Foundation" sheetId="4" r:id="rId4"/>
+    <sheet name="Structural Framing" sheetId="5" r:id="rId5"/>
+    <sheet name="MEP Systems" sheetId="6" r:id="rId6"/>
+    <sheet name="Contingency &amp; Field" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -403,17 +403,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:G8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>SR. NO</v>
       </c>
       <c r="B1" t="str">
-        <v>Type</v>
+        <v>Expense Sub-Category</v>
       </c>
       <c r="C1" t="str">
-        <v>Amount</v>
+        <v>Approved Budget</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Actual Spend</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Variance</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Reconciliation Status</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Line Items &amp; Trades Included</v>
       </c>
     </row>
     <row r="2">
@@ -421,10 +433,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Construction Exp</v>
+        <v>Soft Costs &amp; Engineering</v>
       </c>
       <c r="C2">
-        <v>656154.06</v>
+        <v>343500</v>
+      </c>
+      <c r="D2">
+        <v>343500</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2" t="str">
+        <v>100% Cleared (Draw #1)</v>
+      </c>
+      <c r="G2" t="str">
+        <v>01.01 Architectural Design, 01.02 Structural &amp; Civil Engineering</v>
       </c>
     </row>
     <row r="3">
@@ -432,10 +456,22 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>Labour Exp</v>
+        <v>Municipal &amp; Testing</v>
       </c>
       <c r="C3">
-        <v>73406.5</v>
+        <v>104500</v>
+      </c>
+      <c r="D3">
+        <v>104500</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3" t="str">
+        <v>100% Cleared (Draw #1)</v>
+      </c>
+      <c r="G3" t="str">
+        <v>01.03 Municipal Plan Check &amp; Permits, 01.04 Environmental &amp; Site Survey</v>
       </c>
     </row>
     <row r="4">
@@ -443,10 +479,22 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>Accounting &amp; Legal fee</v>
+        <v>Sitework &amp; Foundation</v>
       </c>
       <c r="C4">
-        <v>1750</v>
+        <v>250300</v>
+      </c>
+      <c r="D4">
+        <v>250300</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="str">
+        <v>100% Cleared (Draw #2)</v>
+      </c>
+      <c r="G4" t="str">
+        <v>02.01 Site Demolition/Excavation, 02.02 Deep Shoring/Piling, 03.01 Foundation Slabs</v>
       </c>
     </row>
     <row r="5">
@@ -454,10 +502,22 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>Bank Fee</v>
+        <v>Structural Framing</v>
       </c>
       <c r="C5">
-        <v>581.51</v>
+        <v>185000</v>
+      </c>
+      <c r="D5">
+        <v>185000</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5" t="str">
+        <v>100% Cleared (Draws #2–#3)</v>
+      </c>
+      <c r="G5" t="str">
+        <v>03.02 Structural Steel Columns, 03.03 Cold-Formed Steel Stud Framing</v>
       </c>
     </row>
     <row r="6">
@@ -465,10 +525,22 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>Municipal Exp</v>
+        <v>MEP Systems</v>
       </c>
       <c r="C6">
-        <v>378</v>
+        <v>180000</v>
+      </c>
+      <c r="D6">
+        <v>175000</v>
+      </c>
+      <c r="E6">
+        <v>-5000</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Active Draw #3 ($5k retainage)</v>
+      </c>
+      <c r="G6" t="str">
+        <v>04.01 Plumbing Rough-In, 04.02 Electrical Service Main, 04.03 HVAC Equipment</v>
       </c>
     </row>
     <row r="7">
@@ -476,541 +548,916 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>Misc Exp</v>
+        <v>Contingency &amp; Field Adjustments</v>
       </c>
       <c r="C7">
-        <v>334649.93</v>
+        <v>3620</v>
+      </c>
+      <c r="D7">
+        <v>8620</v>
+      </c>
+      <c r="E7">
+        <v>5000</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Absorbed in Draw #3</v>
+      </c>
+      <c r="G7" t="str">
+        <v>16.01 Contingency Allocation - Field Pipe Adjustments</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v/>
+      </c>
+      <c r="B8" t="str">
+        <v>Total Reconciled to Bank Statement</v>
+      </c>
+      <c r="C8">
+        <v>1066920</v>
+      </c>
+      <c r="D8">
+        <v>1066920</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8" t="str">
+        <v>100% Verified</v>
+      </c>
+      <c r="G8" t="str">
+        <v>13 Tasks Across Draws #1, #2 &amp; Active Draw #3</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G8"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:J4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Date</v>
+        <v>Line Item</v>
       </c>
       <c r="B1" t="str">
-        <v>Mode</v>
+        <v>Task Description</v>
       </c>
       <c r="C1" t="str">
-        <v>Description</v>
+        <v>Vendor / Counterparty</v>
       </c>
       <c r="D1" t="str">
-        <v>Amount</v>
+        <v>Payment Reference</v>
       </c>
       <c r="E1" t="str">
-        <v/>
+        <v>Target Date</v>
       </c>
       <c r="F1" t="str">
-        <v>Total</v>
-      </c>
-      <c r="G1">
-        <v>656154.06</v>
+        <v>Actual Date</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Approved Budget</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Actual Spend</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Variance</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Payment Status</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <v>45845</v>
+      <c r="A2" t="str">
+        <v>01.01</v>
       </c>
       <c r="B2" t="str">
-        <v>PO-301</v>
+        <v>Architectural Design &amp; Working Drawings</v>
       </c>
       <c r="C2" t="str">
-        <v>Apex Structural Steel Supply &amp; Erect</v>
-      </c>
-      <c r="D2">
-        <v>185000</v>
+        <v>Studio M Architecture</v>
+      </c>
+      <c r="D2" t="str">
+        <v>FedWire #W-4401-A</v>
+      </c>
+      <c r="E2" t="str">
+        <v>May 15, 2025</v>
+      </c>
+      <c r="F2" t="str">
+        <v>May 14, 2025</v>
+      </c>
+      <c r="G2">
+        <v>225000</v>
+      </c>
+      <c r="H2">
+        <v>225000</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Paid • Draw #1 Wire Cleared</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3">
-        <v>45859</v>
+      <c r="A3" t="str">
+        <v>01.02</v>
       </c>
       <c r="B3" t="str">
-        <v>PO-302</v>
+        <v>Structural, MEP &amp; Civil Engineering</v>
       </c>
       <c r="C3" t="str">
-        <v>Carrier Mechanical &amp; HVAC Equipment</v>
-      </c>
-      <c r="D3">
-        <v>95000</v>
+        <v>Apex Engineering Consulting</v>
+      </c>
+      <c r="D3" t="str">
+        <v>FedWire #W-4401-B</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Jun 01, 2025</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Jun 03, 2025</v>
+      </c>
+      <c r="G3">
+        <v>118500</v>
+      </c>
+      <c r="H3">
+        <v>118500</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Paid • Draw #1 Wire Cleared</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4">
-        <v>45890</v>
+      <c r="A4" t="str">
+        <v>Subtotal</v>
       </c>
       <c r="B4" t="str">
-        <v>PO-303</v>
+        <v>Soft Costs &amp; Engineering Total</v>
       </c>
       <c r="C4" t="str">
-        <v>Artisan Architectural Woodwork &amp; Millwork</v>
-      </c>
-      <c r="D4">
-        <v>45000</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>45910</v>
-      </c>
-      <c r="B5" t="str">
-        <v>PO-304</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Peak Engineering &amp; Structural Testing</v>
-      </c>
-      <c r="D5">
-        <v>25000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>45930</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Inv #HV-2025-01</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Horizon HVAC Rough Installation</v>
-      </c>
-      <c r="D6">
-        <v>55000</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <v>45960</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Inv #HV-2025-02</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Horizon Electrical Conduit &amp; Panels</v>
-      </c>
-      <c r="D7">
-        <v>65000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8">
-        <v>45990</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Inv #AC-441</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Apex Framing Supply &amp; Lumbers</v>
-      </c>
-      <c r="D8">
-        <v>78000</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>46010</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Inv #104</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Broadway Framing Package Labor Phase 1</v>
-      </c>
-      <c r="D9">
-        <v>54000</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>46030</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Inv #109</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Broadway Framing Package Labor Phase 2</v>
-      </c>
-      <c r="D10">
-        <v>54154.06</v>
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4">
+        <v>343500</v>
+      </c>
+      <c r="H4">
+        <v>343500</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4" t="str">
+        <v>2 Line Items Verified</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:J4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Date</v>
+        <v>Line Item</v>
       </c>
       <c r="B1" t="str">
-        <v>Mode</v>
+        <v>Task Description</v>
       </c>
       <c r="C1" t="str">
-        <v>Description</v>
+        <v>Vendor / Counterparty</v>
       </c>
       <c r="D1" t="str">
-        <v>Amount</v>
+        <v>Payment Reference</v>
       </c>
       <c r="E1" t="str">
-        <v/>
+        <v>Target Date</v>
       </c>
       <c r="F1" t="str">
-        <v>Total</v>
-      </c>
-      <c r="G1">
-        <v>73406.5</v>
+        <v>Actual Date</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Approved Budget</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Actual Spend</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Variance</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Payment Status</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <v>45846</v>
+      <c r="A2" t="str">
+        <v>01.03</v>
       </c>
       <c r="B2" t="str">
-        <v>Check 1275</v>
+        <v>Municipal Plan Check &amp; Permits</v>
       </c>
       <c r="C2" t="str">
-        <v>Certified Framing Trade Crew</v>
-      </c>
-      <c r="D2">
-        <v>25000</v>
+        <v>City of Newburgh Building Dept</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Check #1092</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Jun 20, 2025</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Jun 18, 2025</v>
+      </c>
+      <c r="G2">
+        <v>54500</v>
+      </c>
+      <c r="H2">
+        <v>54500</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Paid • Certified Check Cleared</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3">
-        <v>45950</v>
+      <c r="A3" t="str">
+        <v>01.04</v>
       </c>
       <c r="B3" t="str">
-        <v>Check 1041</v>
+        <v>Environmental Testing &amp; Site Survey</v>
       </c>
       <c r="C3" t="str">
-        <v>Mechanical Subcontractor Labor</v>
-      </c>
-      <c r="D3">
-        <v>28406.5</v>
+        <v>Hudson Environmental Services</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Check #1094</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Jun 25, 2025</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Jun 24, 2025</v>
+      </c>
+      <c r="G3">
+        <v>50000</v>
+      </c>
+      <c r="H3">
+        <v>50000</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Paid • Corporate Check Cleared</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4">
-        <v>46062</v>
+      <c r="A4" t="str">
+        <v>Subtotal</v>
       </c>
       <c r="B4" t="str">
-        <v>Check 1054</v>
+        <v>Municipal &amp; Testing Total</v>
       </c>
       <c r="C4" t="str">
-        <v>Electrical Rough-in Crew</v>
-      </c>
-      <c r="D4">
-        <v>20000</v>
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4">
+        <v>104500</v>
+      </c>
+      <c r="H4">
+        <v>104500</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4" t="str">
+        <v>2 Line Items Verified</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:J5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Date</v>
+        <v>Line Item</v>
       </c>
       <c r="B1" t="str">
-        <v>Mode</v>
+        <v>Task Description</v>
       </c>
       <c r="C1" t="str">
-        <v>Description</v>
+        <v>Vendor / Counterparty</v>
       </c>
       <c r="D1" t="str">
-        <v>Amount</v>
+        <v>Payment Reference</v>
       </c>
       <c r="E1" t="str">
-        <v/>
+        <v>Target Date</v>
       </c>
       <c r="F1" t="str">
-        <v>Total</v>
-      </c>
-      <c r="G1">
-        <v>1750</v>
+        <v>Actual Date</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Approved Budget</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Actual Spend</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Variance</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Payment Status</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <v>46092</v>
+      <c r="A2" t="str">
+        <v>02.01</v>
       </c>
       <c r="B2" t="str">
-        <v>Debit</v>
+        <v>Site Demolition &amp; Earthwork Excavation</v>
       </c>
       <c r="C2" t="str">
-        <v>Institutional Construction Audit CPA</v>
-      </c>
-      <c r="D2">
-        <v>750</v>
+        <v>Hudson Valley Earthworks LLC</v>
+      </c>
+      <c r="D2" t="str">
+        <v>FedWire #W-4402-A</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Jul 10, 2025</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Jul 12, 2025</v>
+      </c>
+      <c r="G2">
+        <v>85300</v>
+      </c>
+      <c r="H2">
+        <v>85300</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Paid • Draw #2 Wire Cleared</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3">
-        <v>46204</v>
+      <c r="A3" t="str">
+        <v>02.02</v>
       </c>
       <c r="B3" t="str">
-        <v>Debit</v>
+        <v>Deep Foundation, Shoring &amp; Soil Retention</v>
       </c>
       <c r="C3" t="str">
-        <v>Project Legal &amp; Title Review Counsel</v>
-      </c>
-      <c r="D3">
-        <v>1000</v>
+        <v>Tri-State Piling &amp; Shoring</v>
+      </c>
+      <c r="D3" t="str">
+        <v>FedWire #W-4402-B</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Jul 25, 2025</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Jul 28, 2025</v>
+      </c>
+      <c r="G3">
+        <v>50000</v>
+      </c>
+      <c r="H3">
+        <v>50000</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Paid • Draw #2 Wire Cleared</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>03.01</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Reinforced Concrete Core &amp; Foundation Slabs</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Apex Concrete Formwork</v>
+      </c>
+      <c r="D4" t="str">
+        <v>FedWire #W-4402-C</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Aug 15, 2025</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Aug 18, 2025</v>
+      </c>
+      <c r="G4">
+        <v>115000</v>
+      </c>
+      <c r="H4">
+        <v>115000</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Paid • Draw #2 Wire Cleared</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Subtotal</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Sitework &amp; Foundation Total</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5">
+        <v>250300</v>
+      </c>
+      <c r="H5">
+        <v>250300</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5" t="str">
+        <v>3 Line Items Verified</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:J4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Date</v>
+        <v>Line Item</v>
       </c>
       <c r="B1" t="str">
-        <v>Mode</v>
+        <v>Task Description</v>
       </c>
       <c r="C1" t="str">
-        <v>Description</v>
+        <v>Vendor / Counterparty</v>
       </c>
       <c r="D1" t="str">
-        <v>Amount</v>
+        <v>Payment Reference</v>
       </c>
       <c r="E1" t="str">
-        <v/>
+        <v>Target Date</v>
       </c>
       <c r="F1" t="str">
-        <v>Total</v>
-      </c>
-      <c r="G1">
-        <v>581.51</v>
+        <v>Actual Date</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Approved Budget</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Actual Spend</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Variance</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Payment Status</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <v>45751</v>
+      <c r="A2" t="str">
+        <v>03.02</v>
       </c>
       <c r="B2" t="str">
-        <v>Debit</v>
+        <v>Structural Steel Columns &amp; Moment Connections</v>
       </c>
       <c r="C2" t="str">
-        <v>Commercial Wire Transfer Fee</v>
-      </c>
-      <c r="D2">
-        <v>20</v>
+        <v>Broadway Structural Framing</v>
+      </c>
+      <c r="D2" t="str">
+        <v>FedWire #W-4402-D</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Sep 01, 2025</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Sep 25, 2025</v>
+      </c>
+      <c r="G2">
+        <v>69700</v>
+      </c>
+      <c r="H2">
+        <v>69700</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Paid • Draw #2 Wire Cleared</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3">
-        <v>45768</v>
+      <c r="A3" t="str">
+        <v>03.03</v>
       </c>
       <c r="B3" t="str">
-        <v>Debit</v>
+        <v>Cold-Formed Light Gauge Steel Stud Framing</v>
       </c>
       <c r="C3" t="str">
-        <v>Commercial Wire Transfer Fee</v>
-      </c>
-      <c r="D3">
-        <v>20</v>
+        <v>Empire Framing Contractors</v>
+      </c>
+      <c r="D3" t="str">
+        <v>FedWire #W-4403-A</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Sep 20, 2025</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Oct 05, 2025</v>
+      </c>
+      <c r="G3">
+        <v>115300</v>
+      </c>
+      <c r="H3">
+        <v>115300</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Paid • Draw #3 Wire Cleared</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4">
-        <v>45770</v>
+      <c r="A4" t="str">
+        <v>Subtotal</v>
       </c>
       <c r="B4" t="str">
-        <v>Debit</v>
+        <v>Structural Framing Total</v>
       </c>
       <c r="C4" t="str">
-        <v>Escrow Disbursement Maintenance Fee</v>
-      </c>
-      <c r="D4">
-        <v>541.51</v>
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4">
+        <v>185000</v>
+      </c>
+      <c r="H4">
+        <v>185000</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4" t="str">
+        <v>2 Line Items Verified</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:J5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Date</v>
+        <v>Line Item</v>
       </c>
       <c r="B1" t="str">
-        <v>Mode</v>
+        <v>Task Description</v>
       </c>
       <c r="C1" t="str">
-        <v>Description</v>
+        <v>Vendor / Counterparty</v>
       </c>
       <c r="D1" t="str">
-        <v>Amount</v>
+        <v>Payment Reference</v>
       </c>
       <c r="E1" t="str">
-        <v/>
+        <v>Target Date</v>
       </c>
       <c r="F1" t="str">
-        <v>Total</v>
-      </c>
-      <c r="G1">
-        <v>378</v>
+        <v>Actual Date</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Approved Budget</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Actual Spend</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Variance</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Payment Status</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <v>45841</v>
+      <c r="A2" t="str">
+        <v>04.01</v>
       </c>
       <c r="B2" t="str">
-        <v>Debit</v>
+        <v>Plumbing Waste, Vent &amp; Water Distribution</v>
       </c>
       <c r="C2" t="str">
-        <v>Municipal Department of Buildings Plan Filing</v>
-      </c>
-      <c r="D2">
-        <v>126</v>
+        <v>Metropolitan Mechanical &amp; Plumbing</v>
+      </c>
+      <c r="D2" t="str">
+        <v>FedWire #W-4403-B</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Oct 01, 2025</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Oct 10, 2025</v>
+      </c>
+      <c r="G2">
+        <v>65000</v>
+      </c>
+      <c r="H2">
+        <v>65000</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Paid • Draw #3 Wire Cleared</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3">
-        <v>46071</v>
+      <c r="A3" t="str">
+        <v>04.02</v>
       </c>
       <c r="B3" t="str">
-        <v>Debit</v>
+        <v>Electrical Service Main &amp; Conduit Rough-Ins</v>
       </c>
       <c r="C3" t="str">
-        <v>Municipal Water &amp; Sewer Inspection</v>
-      </c>
-      <c r="D3">
-        <v>126</v>
+        <v>Apex Power &amp; Electrical LLC</v>
+      </c>
+      <c r="D3" t="str">
+        <v>FedWire #W-4403-C</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Oct 15, 2025</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Oct 18, 2025</v>
+      </c>
+      <c r="G3">
+        <v>75000</v>
+      </c>
+      <c r="H3">
+        <v>75000</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Paid • Draw #3 Wire Cleared</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4">
-        <v>46077</v>
+      <c r="A4" t="str">
+        <v>04.03</v>
       </c>
       <c r="B4" t="str">
-        <v>Debit</v>
+        <v>HVAC Equipment &amp; Duct Distribution</v>
       </c>
       <c r="C4" t="str">
-        <v>Municipal Environmental Sign-off</v>
-      </c>
-      <c r="D4">
-        <v>126</v>
+        <v>Carrier Climate Systems</v>
+      </c>
+      <c r="D4" t="str">
+        <v>FedWire #W-4403-D</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Oct 20, 2025</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Oct 24, 2025</v>
+      </c>
+      <c r="G4">
+        <v>40000</v>
+      </c>
+      <c r="H4">
+        <v>35000</v>
+      </c>
+      <c r="I4">
+        <v>-5000</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Active Spend • $5k Retainage Held</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Subtotal</v>
+      </c>
+      <c r="B5" t="str">
+        <v>MEP Systems Total</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5">
+        <v>180000</v>
+      </c>
+      <c r="H5">
+        <v>175000</v>
+      </c>
+      <c r="I5">
+        <v>-5000</v>
+      </c>
+      <c r="J5" t="str">
+        <v>3 Line Items Verified</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:J3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Date</v>
+        <v>Line Item</v>
       </c>
       <c r="B1" t="str">
-        <v>Mode</v>
+        <v>Task Description</v>
       </c>
       <c r="C1" t="str">
-        <v>Description</v>
+        <v>Vendor / Counterparty</v>
       </c>
       <c r="D1" t="str">
-        <v>Amount</v>
+        <v>Payment Reference</v>
       </c>
       <c r="E1" t="str">
-        <v/>
+        <v>Target Date</v>
       </c>
       <c r="F1" t="str">
-        <v>Total</v>
-      </c>
-      <c r="G1">
-        <v>334649.93</v>
+        <v>Actual Date</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Approved Budget</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Actual Spend</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Variance</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Payment Status</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <v>45820</v>
+      <c r="A2" t="str">
+        <v>16.01</v>
       </c>
       <c r="B2" t="str">
-        <v>Check 1001</v>
+        <v>Contingency Allocation - Field Pipe Adjustments</v>
       </c>
       <c r="C2" t="str">
-        <v>Jobsite Facilities, Office Trailer &amp; Security</v>
-      </c>
-      <c r="D2">
-        <v>114649.93</v>
+        <v>Trade Contractors Allocation</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Debit #D-8821</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Oct 22, 2025</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Oct 25, 2025</v>
+      </c>
+      <c r="G2">
+        <v>3620</v>
+      </c>
+      <c r="H2">
+        <v>8620</v>
+      </c>
+      <c r="I2">
+        <v>5000</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Paid • Contingency Absorbed</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3">
-        <v>45900</v>
+      <c r="A3" t="str">
+        <v>Subtotal</v>
       </c>
       <c r="B3" t="str">
-        <v>Debit</v>
+        <v>Contingency Total</v>
       </c>
       <c r="C3" t="str">
-        <v>Temporary Site Utilities &amp; Power Hookups</v>
-      </c>
-      <c r="D3">
-        <v>120000</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>46000</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Wire</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Field Superintendent &amp; General Conditions Carry</v>
-      </c>
-      <c r="D4">
-        <v>100000</v>
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3">
+        <v>3620</v>
+      </c>
+      <c r="H3">
+        <v>8620</v>
+      </c>
+      <c r="I3">
+        <v>5000</v>
+      </c>
+      <c r="J3" t="str">
+        <v>1 Line Item Verified</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(demo-data): update expense tracker subcategories and sheet tabs
</commit_message>
<xml_diff>
--- a/frontend/public/sample-docs/73 Broadway - Expense Tracker.xlsx
+++ b/frontend/public/sample-docs/73 Broadway - Expense Tracker.xlsx
@@ -4,12 +4,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Total Expenses" sheetId="1" r:id="rId1"/>
-    <sheet name="Soft Costs" sheetId="2" r:id="rId2"/>
-    <sheet name="Municipal &amp; Permits" sheetId="3" r:id="rId3"/>
-    <sheet name="Sitework &amp; Foundation" sheetId="4" r:id="rId4"/>
-    <sheet name="Structural Framing" sheetId="5" r:id="rId5"/>
-    <sheet name="MEP Systems" sheetId="6" r:id="rId6"/>
-    <sheet name="Contingency &amp; Field" sheetId="7" r:id="rId7"/>
+    <sheet name="Construction Expense" sheetId="2" r:id="rId2"/>
+    <sheet name="Labour Expense" sheetId="3" r:id="rId3"/>
+    <sheet name="Accounts &amp; Legal Fees" sheetId="4" r:id="rId4"/>
+    <sheet name="Bank Fees" sheetId="5" r:id="rId5"/>
+    <sheet name="Municipal Expense" sheetId="6" r:id="rId6"/>
+    <sheet name="Miscellaneous Expense" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -433,22 +433,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Soft Costs &amp; Engineering</v>
+        <v>Construction Expense</v>
       </c>
       <c r="C2">
-        <v>343500</v>
+        <v>250300</v>
       </c>
       <c r="D2">
-        <v>343500</v>
+        <v>250300</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2" t="str">
-        <v>100% Cleared (Draw #1)</v>
+        <v>100% Cleared (Draw #2)</v>
       </c>
       <c r="G2" t="str">
-        <v>01.01 Architectural Design, 01.02 Structural &amp; Civil Engineering</v>
+        <v>02.01 Site Demolition/Excavation, 02.02 Deep Shoring/Piling, 03.01 Foundation Slabs</v>
       </c>
     </row>
     <row r="3">
@@ -456,22 +456,22 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>Municipal &amp; Testing</v>
+        <v>Labour Expense</v>
       </c>
       <c r="C3">
-        <v>104500</v>
+        <v>185000</v>
       </c>
       <c r="D3">
-        <v>104500</v>
+        <v>185000</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="F3" t="str">
-        <v>100% Cleared (Draw #1)</v>
+        <v>100% Cleared (Draws #2–#3)</v>
       </c>
       <c r="G3" t="str">
-        <v>01.03 Municipal Plan Check &amp; Permits, 01.04 Environmental &amp; Site Survey</v>
+        <v>03.02 Structural Steel Columns, 03.03 Cold-Formed Steel Stud Framing</v>
       </c>
     </row>
     <row r="4">
@@ -479,22 +479,22 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>Sitework &amp; Foundation</v>
+        <v>Accounts &amp; Legal Fees</v>
       </c>
       <c r="C4">
-        <v>250300</v>
+        <v>343500</v>
       </c>
       <c r="D4">
-        <v>250300</v>
+        <v>343500</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4" t="str">
-        <v>100% Cleared (Draw #2)</v>
+        <v>100% Cleared (Draw #1)</v>
       </c>
       <c r="G4" t="str">
-        <v>02.01 Site Demolition/Excavation, 02.02 Deep Shoring/Piling, 03.01 Foundation Slabs</v>
+        <v>01.01 Architectural Design, 01.02 Structural &amp; Civil Engineering</v>
       </c>
     </row>
     <row r="5">
@@ -502,22 +502,22 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>Structural Framing</v>
+        <v>Bank Fees</v>
       </c>
       <c r="C5">
-        <v>185000</v>
+        <v>180000</v>
       </c>
       <c r="D5">
-        <v>185000</v>
+        <v>175000</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>-5000</v>
       </c>
       <c r="F5" t="str">
-        <v>100% Cleared (Draws #2–#3)</v>
+        <v>Active Draw #3 ($5k retainage)</v>
       </c>
       <c r="G5" t="str">
-        <v>03.02 Structural Steel Columns, 03.03 Cold-Formed Steel Stud Framing</v>
+        <v>04.01 Plumbing Rough-In, 04.02 Electrical Service Main, 04.03 HVAC Equipment</v>
       </c>
     </row>
     <row r="6">
@@ -525,22 +525,22 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>MEP Systems</v>
+        <v>Municipal Expense</v>
       </c>
       <c r="C6">
-        <v>180000</v>
+        <v>104500</v>
       </c>
       <c r="D6">
-        <v>175000</v>
+        <v>104500</v>
       </c>
       <c r="E6">
-        <v>-5000</v>
+        <v>0</v>
       </c>
       <c r="F6" t="str">
-        <v>Active Draw #3 ($5k retainage)</v>
+        <v>100% Cleared (Draw #1)</v>
       </c>
       <c r="G6" t="str">
-        <v>04.01 Plumbing Rough-In, 04.02 Electrical Service Main, 04.03 HVAC Equipment</v>
+        <v>01.03 Municipal Plan Check &amp; Permits, 01.04 Environmental &amp; Site Survey</v>
       </c>
     </row>
     <row r="7">
@@ -548,7 +548,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>Contingency &amp; Field Adjustments</v>
+        <v>Miscellaneous Expense</v>
       </c>
       <c r="C7">
         <v>3620</v>
@@ -598,7 +598,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -634,103 +634,135 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>01.01</v>
+        <v>02.01</v>
       </c>
       <c r="B2" t="str">
-        <v>Architectural Design &amp; Working Drawings</v>
+        <v>Site Demolition &amp; Earthwork Excavation</v>
       </c>
       <c r="C2" t="str">
-        <v>Studio M Architecture</v>
+        <v>Hudson Valley Earthworks LLC</v>
       </c>
       <c r="D2" t="str">
-        <v>FedWire #W-4401-A</v>
+        <v>FedWire #W-4402-A</v>
       </c>
       <c r="E2" t="str">
-        <v>May 15, 2025</v>
+        <v>Jul 10, 2025</v>
       </c>
       <c r="F2" t="str">
-        <v>May 14, 2025</v>
+        <v>Jul 12, 2025</v>
       </c>
       <c r="G2">
-        <v>225000</v>
+        <v>85300</v>
       </c>
       <c r="H2">
-        <v>225000</v>
+        <v>85300</v>
       </c>
       <c r="I2">
         <v>0</v>
       </c>
       <c r="J2" t="str">
-        <v>Paid • Draw #1 Wire Cleared</v>
+        <v>Paid • Draw #2 Wire Cleared</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>01.02</v>
+        <v>02.02</v>
       </c>
       <c r="B3" t="str">
-        <v>Structural, MEP &amp; Civil Engineering</v>
+        <v>Deep Foundation, Shoring &amp; Soil Retention</v>
       </c>
       <c r="C3" t="str">
-        <v>Apex Engineering Consulting</v>
+        <v>Tri-State Piling &amp; Shoring</v>
       </c>
       <c r="D3" t="str">
-        <v>FedWire #W-4401-B</v>
+        <v>FedWire #W-4402-B</v>
       </c>
       <c r="E3" t="str">
-        <v>Jun 01, 2025</v>
+        <v>Jul 25, 2025</v>
       </c>
       <c r="F3" t="str">
-        <v>Jun 03, 2025</v>
+        <v>Jul 28, 2025</v>
       </c>
       <c r="G3">
-        <v>118500</v>
+        <v>50000</v>
       </c>
       <c r="H3">
-        <v>118500</v>
+        <v>50000</v>
       </c>
       <c r="I3">
         <v>0</v>
       </c>
       <c r="J3" t="str">
-        <v>Paid • Draw #1 Wire Cleared</v>
+        <v>Paid • Draw #2 Wire Cleared</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>03.01</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Reinforced Concrete Core &amp; Foundation Slabs</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Apex Concrete Formwork</v>
+      </c>
+      <c r="D4" t="str">
+        <v>FedWire #W-4402-C</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Aug 15, 2025</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Aug 18, 2025</v>
+      </c>
+      <c r="G4">
+        <v>115000</v>
+      </c>
+      <c r="H4">
+        <v>115000</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Paid • Draw #2 Wire Cleared</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
         <v>Subtotal</v>
       </c>
-      <c r="B4" t="str">
-        <v>Soft Costs &amp; Engineering Total</v>
-      </c>
-      <c r="C4" t="str">
-        <v/>
-      </c>
-      <c r="D4" t="str">
-        <v/>
-      </c>
-      <c r="E4" t="str">
-        <v/>
-      </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
-      <c r="G4">
-        <v>343500</v>
-      </c>
-      <c r="H4">
-        <v>343500</v>
-      </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4" t="str">
-        <v>2 Line Items Verified</v>
+      <c r="B5" t="str">
+        <v>Construction Expense Total</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5">
+        <v>250300</v>
+      </c>
+      <c r="H5">
+        <v>250300</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5" t="str">
+        <v>3 Line Items Verified</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -773,66 +805,66 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>01.03</v>
+        <v>03.02</v>
       </c>
       <c r="B2" t="str">
-        <v>Municipal Plan Check &amp; Permits</v>
+        <v>Structural Steel Columns &amp; Moment Connections</v>
       </c>
       <c r="C2" t="str">
-        <v>City of Newburgh Building Dept</v>
+        <v>Broadway Structural Framing</v>
       </c>
       <c r="D2" t="str">
-        <v>Check #1092</v>
+        <v>FedWire #W-4402-D</v>
       </c>
       <c r="E2" t="str">
-        <v>Jun 20, 2025</v>
+        <v>Sep 01, 2025</v>
       </c>
       <c r="F2" t="str">
-        <v>Jun 18, 2025</v>
+        <v>Sep 25, 2025</v>
       </c>
       <c r="G2">
-        <v>54500</v>
+        <v>69700</v>
       </c>
       <c r="H2">
-        <v>54500</v>
+        <v>69700</v>
       </c>
       <c r="I2">
         <v>0</v>
       </c>
       <c r="J2" t="str">
-        <v>Paid • Certified Check Cleared</v>
+        <v>Paid • Draw #2 Wire Cleared</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>01.04</v>
+        <v>03.03</v>
       </c>
       <c r="B3" t="str">
-        <v>Environmental Testing &amp; Site Survey</v>
+        <v>Cold-Formed Light Gauge Steel Stud Framing</v>
       </c>
       <c r="C3" t="str">
-        <v>Hudson Environmental Services</v>
+        <v>Empire Framing Contractors</v>
       </c>
       <c r="D3" t="str">
-        <v>Check #1094</v>
+        <v>FedWire #W-4403-A</v>
       </c>
       <c r="E3" t="str">
-        <v>Jun 25, 2025</v>
+        <v>Sep 20, 2025</v>
       </c>
       <c r="F3" t="str">
-        <v>Jun 24, 2025</v>
+        <v>Oct 05, 2025</v>
       </c>
       <c r="G3">
-        <v>50000</v>
+        <v>115300</v>
       </c>
       <c r="H3">
-        <v>50000</v>
+        <v>115300</v>
       </c>
       <c r="I3">
         <v>0</v>
       </c>
       <c r="J3" t="str">
-        <v>Paid • Corporate Check Cleared</v>
+        <v>Paid • Draw #3 Wire Cleared</v>
       </c>
     </row>
     <row r="4">
@@ -840,7 +872,7 @@
         <v>Subtotal</v>
       </c>
       <c r="B4" t="str">
-        <v>Municipal &amp; Testing Total</v>
+        <v>Labour Expense Total</v>
       </c>
       <c r="C4" t="str">
         <v/>
@@ -855,10 +887,10 @@
         <v/>
       </c>
       <c r="G4">
-        <v>104500</v>
+        <v>185000</v>
       </c>
       <c r="H4">
-        <v>104500</v>
+        <v>185000</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -876,6 +908,145 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Line Item</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Task Description</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Vendor / Counterparty</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Payment Reference</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Target Date</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Actual Date</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Approved Budget</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Actual Spend</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Variance</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Payment Status</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>01.01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Architectural Design &amp; Working Drawings</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Studio M Architecture</v>
+      </c>
+      <c r="D2" t="str">
+        <v>FedWire #W-4401-A</v>
+      </c>
+      <c r="E2" t="str">
+        <v>May 15, 2025</v>
+      </c>
+      <c r="F2" t="str">
+        <v>May 14, 2025</v>
+      </c>
+      <c r="G2">
+        <v>225000</v>
+      </c>
+      <c r="H2">
+        <v>225000</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Paid • Draw #1 Wire Cleared</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>01.02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Structural, MEP &amp; Civil Engineering</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Apex Engineering Consulting</v>
+      </c>
+      <c r="D3" t="str">
+        <v>FedWire #W-4401-B</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Jun 01, 2025</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Jun 03, 2025</v>
+      </c>
+      <c r="G3">
+        <v>118500</v>
+      </c>
+      <c r="H3">
+        <v>118500</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Paid • Draw #1 Wire Cleared</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Subtotal</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Accounts &amp; Legal Fees Total</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4">
+        <v>343500</v>
+      </c>
+      <c r="H4">
+        <v>343500</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4" t="str">
+        <v>2 Line Items Verified</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J5"/>
   <sheetData>
     <row r="1">
@@ -912,98 +1083,98 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>02.01</v>
+        <v>04.01</v>
       </c>
       <c r="B2" t="str">
-        <v>Site Demolition &amp; Earthwork Excavation</v>
+        <v>Plumbing Waste, Vent &amp; Water Distribution</v>
       </c>
       <c r="C2" t="str">
-        <v>Hudson Valley Earthworks LLC</v>
+        <v>Metropolitan Mechanical &amp; Plumbing</v>
       </c>
       <c r="D2" t="str">
-        <v>FedWire #W-4402-A</v>
+        <v>FedWire #W-4403-B</v>
       </c>
       <c r="E2" t="str">
-        <v>Jul 10, 2025</v>
+        <v>Oct 01, 2025</v>
       </c>
       <c r="F2" t="str">
-        <v>Jul 12, 2025</v>
+        <v>Oct 10, 2025</v>
       </c>
       <c r="G2">
-        <v>85300</v>
+        <v>65000</v>
       </c>
       <c r="H2">
-        <v>85300</v>
+        <v>65000</v>
       </c>
       <c r="I2">
         <v>0</v>
       </c>
       <c r="J2" t="str">
-        <v>Paid • Draw #2 Wire Cleared</v>
+        <v>Paid • Draw #3 Wire Cleared</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>02.02</v>
+        <v>04.02</v>
       </c>
       <c r="B3" t="str">
-        <v>Deep Foundation, Shoring &amp; Soil Retention</v>
+        <v>Electrical Service Main &amp; Conduit Rough-Ins</v>
       </c>
       <c r="C3" t="str">
-        <v>Tri-State Piling &amp; Shoring</v>
+        <v>Apex Power &amp; Electrical LLC</v>
       </c>
       <c r="D3" t="str">
-        <v>FedWire #W-4402-B</v>
+        <v>FedWire #W-4403-C</v>
       </c>
       <c r="E3" t="str">
-        <v>Jul 25, 2025</v>
+        <v>Oct 15, 2025</v>
       </c>
       <c r="F3" t="str">
-        <v>Jul 28, 2025</v>
+        <v>Oct 18, 2025</v>
       </c>
       <c r="G3">
-        <v>50000</v>
+        <v>75000</v>
       </c>
       <c r="H3">
-        <v>50000</v>
+        <v>75000</v>
       </c>
       <c r="I3">
         <v>0</v>
       </c>
       <c r="J3" t="str">
-        <v>Paid • Draw #2 Wire Cleared</v>
+        <v>Paid • Draw #3 Wire Cleared</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>03.01</v>
+        <v>04.03</v>
       </c>
       <c r="B4" t="str">
-        <v>Reinforced Concrete Core &amp; Foundation Slabs</v>
+        <v>HVAC Equipment &amp; Duct Distribution</v>
       </c>
       <c r="C4" t="str">
-        <v>Apex Concrete Formwork</v>
+        <v>Carrier Climate Systems</v>
       </c>
       <c r="D4" t="str">
-        <v>FedWire #W-4402-C</v>
+        <v>FedWire #W-4403-D</v>
       </c>
       <c r="E4" t="str">
-        <v>Aug 15, 2025</v>
+        <v>Oct 20, 2025</v>
       </c>
       <c r="F4" t="str">
-        <v>Aug 18, 2025</v>
+        <v>Oct 24, 2025</v>
       </c>
       <c r="G4">
-        <v>115000</v>
+        <v>40000</v>
       </c>
       <c r="H4">
-        <v>115000</v>
+        <v>35000</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>-5000</v>
       </c>
       <c r="J4" t="str">
-        <v>Paid • Draw #2 Wire Cleared</v>
+        <v>Active Spend • $5k Retainage Held</v>
       </c>
     </row>
     <row r="5">
@@ -1011,7 +1182,7 @@
         <v>Subtotal</v>
       </c>
       <c r="B5" t="str">
-        <v>Sitework &amp; Foundation Total</v>
+        <v>Bank Fees Total</v>
       </c>
       <c r="C5" t="str">
         <v/>
@@ -1026,13 +1197,13 @@
         <v/>
       </c>
       <c r="G5">
-        <v>250300</v>
+        <v>180000</v>
       </c>
       <c r="H5">
-        <v>250300</v>
+        <v>175000</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>-5000</v>
       </c>
       <c r="J5" t="str">
         <v>3 Line Items Verified</v>
@@ -1045,7 +1216,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J4"/>
   <sheetData>
@@ -1083,66 +1254,66 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>03.02</v>
+        <v>01.03</v>
       </c>
       <c r="B2" t="str">
-        <v>Structural Steel Columns &amp; Moment Connections</v>
+        <v>Municipal Plan Check &amp; Permits</v>
       </c>
       <c r="C2" t="str">
-        <v>Broadway Structural Framing</v>
+        <v>City of Newburgh Building Dept</v>
       </c>
       <c r="D2" t="str">
-        <v>FedWire #W-4402-D</v>
+        <v>Check #1092</v>
       </c>
       <c r="E2" t="str">
-        <v>Sep 01, 2025</v>
+        <v>Jun 20, 2025</v>
       </c>
       <c r="F2" t="str">
-        <v>Sep 25, 2025</v>
+        <v>Jun 18, 2025</v>
       </c>
       <c r="G2">
-        <v>69700</v>
+        <v>54500</v>
       </c>
       <c r="H2">
-        <v>69700</v>
+        <v>54500</v>
       </c>
       <c r="I2">
         <v>0</v>
       </c>
       <c r="J2" t="str">
-        <v>Paid • Draw #2 Wire Cleared</v>
+        <v>Paid • Certified Check Cleared</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>03.03</v>
+        <v>01.04</v>
       </c>
       <c r="B3" t="str">
-        <v>Cold-Formed Light Gauge Steel Stud Framing</v>
+        <v>Environmental Testing &amp; Site Survey</v>
       </c>
       <c r="C3" t="str">
-        <v>Empire Framing Contractors</v>
+        <v>Hudson Environmental Services</v>
       </c>
       <c r="D3" t="str">
-        <v>FedWire #W-4403-A</v>
+        <v>Check #1094</v>
       </c>
       <c r="E3" t="str">
-        <v>Sep 20, 2025</v>
+        <v>Jun 25, 2025</v>
       </c>
       <c r="F3" t="str">
-        <v>Oct 05, 2025</v>
+        <v>Jun 24, 2025</v>
       </c>
       <c r="G3">
-        <v>115300</v>
+        <v>50000</v>
       </c>
       <c r="H3">
-        <v>115300</v>
+        <v>50000</v>
       </c>
       <c r="I3">
         <v>0</v>
       </c>
       <c r="J3" t="str">
-        <v>Paid • Draw #3 Wire Cleared</v>
+        <v>Paid • Corporate Check Cleared</v>
       </c>
     </row>
     <row r="4">
@@ -1150,7 +1321,7 @@
         <v>Subtotal</v>
       </c>
       <c r="B4" t="str">
-        <v>Structural Framing Total</v>
+        <v>Municipal Expense Total</v>
       </c>
       <c r="C4" t="str">
         <v/>
@@ -1165,10 +1336,10 @@
         <v/>
       </c>
       <c r="G4">
-        <v>185000</v>
+        <v>104500</v>
       </c>
       <c r="H4">
-        <v>185000</v>
+        <v>104500</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -1180,177 +1351,6 @@
   </sheetData>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J5"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Line Item</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Task Description</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Vendor / Counterparty</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Payment Reference</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Target Date</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Actual Date</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Approved Budget</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Actual Spend</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Variance</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Payment Status</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>04.01</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Plumbing Waste, Vent &amp; Water Distribution</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Metropolitan Mechanical &amp; Plumbing</v>
-      </c>
-      <c r="D2" t="str">
-        <v>FedWire #W-4403-B</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Oct 01, 2025</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Oct 10, 2025</v>
-      </c>
-      <c r="G2">
-        <v>65000</v>
-      </c>
-      <c r="H2">
-        <v>65000</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2" t="str">
-        <v>Paid • Draw #3 Wire Cleared</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>04.02</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Electrical Service Main &amp; Conduit Rough-Ins</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Apex Power &amp; Electrical LLC</v>
-      </c>
-      <c r="D3" t="str">
-        <v>FedWire #W-4403-C</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Oct 15, 2025</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Oct 18, 2025</v>
-      </c>
-      <c r="G3">
-        <v>75000</v>
-      </c>
-      <c r="H3">
-        <v>75000</v>
-      </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
-      <c r="J3" t="str">
-        <v>Paid • Draw #3 Wire Cleared</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>04.03</v>
-      </c>
-      <c r="B4" t="str">
-        <v>HVAC Equipment &amp; Duct Distribution</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Carrier Climate Systems</v>
-      </c>
-      <c r="D4" t="str">
-        <v>FedWire #W-4403-D</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Oct 20, 2025</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Oct 24, 2025</v>
-      </c>
-      <c r="G4">
-        <v>40000</v>
-      </c>
-      <c r="H4">
-        <v>35000</v>
-      </c>
-      <c r="I4">
-        <v>-5000</v>
-      </c>
-      <c r="J4" t="str">
-        <v>Active Spend • $5k Retainage Held</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Subtotal</v>
-      </c>
-      <c r="B5" t="str">
-        <v>MEP Systems Total</v>
-      </c>
-      <c r="C5" t="str">
-        <v/>
-      </c>
-      <c r="D5" t="str">
-        <v/>
-      </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
-      <c r="F5" t="str">
-        <v/>
-      </c>
-      <c r="G5">
-        <v>180000</v>
-      </c>
-      <c r="H5">
-        <v>175000</v>
-      </c>
-      <c r="I5">
-        <v>-5000</v>
-      </c>
-      <c r="J5" t="str">
-        <v>3 Line Items Verified</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1428,7 +1428,7 @@
         <v>Subtotal</v>
       </c>
       <c r="B3" t="str">
-        <v>Contingency Total</v>
+        <v>Miscellaneous Expense Total</v>
       </c>
       <c r="C3" t="str">
         <v/>

</xml_diff>

<commit_message>
feat(control-center): rename target and actual dates to start and completion dates in spend comparison
- Update column headers in MetricDetailPanel and AmountSourceModal to Start Date and Completion Date

- Update generate-expense-tracker-xlsx script and synchronized spreadsheets
</commit_message>
<xml_diff>
--- a/frontend/public/sample-docs/73 Broadway - Expense Tracker.xlsx
+++ b/frontend/public/sample-docs/73 Broadway - Expense Tracker.xlsx
@@ -614,10 +614,10 @@
         <v>Payment Reference</v>
       </c>
       <c r="E1" t="str">
-        <v>Target Date</v>
+        <v>Start Date</v>
       </c>
       <c r="F1" t="str">
-        <v>Actual Date</v>
+        <v>Completion Date</v>
       </c>
       <c r="G1" t="str">
         <v>Approved Budget</v>
@@ -785,10 +785,10 @@
         <v>Payment Reference</v>
       </c>
       <c r="E1" t="str">
-        <v>Target Date</v>
+        <v>Start Date</v>
       </c>
       <c r="F1" t="str">
-        <v>Actual Date</v>
+        <v>Completion Date</v>
       </c>
       <c r="G1" t="str">
         <v>Approved Budget</v>
@@ -924,10 +924,10 @@
         <v>Payment Reference</v>
       </c>
       <c r="E1" t="str">
-        <v>Target Date</v>
+        <v>Start Date</v>
       </c>
       <c r="F1" t="str">
-        <v>Actual Date</v>
+        <v>Completion Date</v>
       </c>
       <c r="G1" t="str">
         <v>Approved Budget</v>
@@ -1063,10 +1063,10 @@
         <v>Payment Reference</v>
       </c>
       <c r="E1" t="str">
-        <v>Target Date</v>
+        <v>Start Date</v>
       </c>
       <c r="F1" t="str">
-        <v>Actual Date</v>
+        <v>Completion Date</v>
       </c>
       <c r="G1" t="str">
         <v>Approved Budget</v>
@@ -1234,10 +1234,10 @@
         <v>Payment Reference</v>
       </c>
       <c r="E1" t="str">
-        <v>Target Date</v>
+        <v>Start Date</v>
       </c>
       <c r="F1" t="str">
-        <v>Actual Date</v>
+        <v>Completion Date</v>
       </c>
       <c r="G1" t="str">
         <v>Approved Budget</v>
@@ -1373,10 +1373,10 @@
         <v>Payment Reference</v>
       </c>
       <c r="E1" t="str">
-        <v>Target Date</v>
+        <v>Start Date</v>
       </c>
       <c r="F1" t="str">
-        <v>Actual Date</v>
+        <v>Completion Date</v>
       </c>
       <c r="G1" t="str">
         <v>Approved Budget</v>

</xml_diff>